<commit_message>
Epic 9 tracker: add Sprint 9 (Hero v2 layered parallax + video mockup)
Sprint 9 covers the recent hero rebuild shipped in commit 15b51cc:
three-plane depth composition (sunset bg + product-tour video card in
the middle + desk foreground plane), per-layer parallax curves + blur,
right-to-left marquee trust band, autoplay hardened, nav visible on
hero, and the reveal-class-override bug fix that was silently killing
video-card parallax.

- Cover: appended Sprint 9 block with Scope / Why / Status / Supersedes
  (S9 replaces S5-06 hero background video and S6-03 pin+blur behaviour)
- Dashboard: Sprint 9 row = 15/15 Done. Epic rollup 70/74 (95%).
- Backlog: 15 rows U9-09.1 .. U9-09.15, each shipped in the same commit.
- Master Tracker: Epic 9 row updated to 70/74. Rollup recomputed to
  334/457 (73%). No other epic row touched.

Sprint 8 (open items) still open as before -- FAQ direction, logo colour
mismatch, GitHub Pages hosting, post-Pages production deployment.
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic9_Landing_Page.xlsx
+++ b/docs/DecisionOS_Epic9_Landing_Page.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1023,6 +1023,70 @@
     <row r="54">
       <c r="A54" s="18" t="inlineStr"/>
       <c r="B54" s="18" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="18" t="inlineStr"/>
+      <c r="B55" s="18" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="inlineStr">
+        <is>
+          <t>&gt;&gt;&gt; Sprint 9 -- Hero v2 (layered parallax + video mockup)</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="18" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>Rebuilt the hero from a static single-photo composition into a three-plane layered scene. Background (hero-bg.jpg -- sunset valley), middle plane (copy + video card + trust band), foreground (hero-fg.webp -- desk with laptop / notebook / glass, alpha-preserved). Replaced the 6-card metric grid with a single curved card playing a 10-second product-tour video (hero-mockup.webm + .mp4 fallback), top-cropped to hide the browser Chrome. Trust band lifted from the hero bottom into a mid-band marquee (right-to-left seamless loop, fade-edge masks, 780px contained width). Per-layer parallax on scroll -- each of the six visible elements counter-translates at its own rate (bg 30% apparent speed, fg 100%, copy 70%, video card 68%, dex 60%, trust band 55%) with an independent blur curve. Nav bar always visible on the hero (removed hide-until-scroll behaviour). Dex bubble and scroll cue removed. Autoplay hardened with 250ms poll + first-interaction fallback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="18" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>The static amber-wall hero didn't communicate what DecisionOS actually IS -- it read as a motivational poster, not a product. A layered scene with an in-frame video demo tells the story in the first paint, and the parallax gives the composition three-dimensional depth without asking the visitor to interact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="18" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>Done -- shipped 2026-08-28 (commit 15b51cc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="18" t="inlineStr"/>
+      <c r="B60" s="18" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="18" t="inlineStr">
+        <is>
+          <t>Supersedes</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>S5-06 (hero background video, added then reverted) and S6-03 (sticky-pin hero + blur on next-section overlap) are effectively replaced by S9. The pin-and-recede model was rebuilt as per-layer lag parallax with each plane parallaxing independently as the hero scrolls up.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1035,7 +1099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1076,7 +1140,7 @@
     <row r="3">
       <c r="A3" s="20" t="inlineStr">
         <is>
-          <t>Epic 9 status: IN PROGRESS. Sprints 1-7 shipped (55/59, 93%). Sprint 8 (Open Items) tracks FAQ sign-off, logo colour mismatch, GitHub Pages hosting, and post-Pages production deployment.</t>
+          <t>Epic 9 status: IN PROGRESS. Sprints 1-7 shipped (55/59). S9 -- Hero v2 layered parallax + video mockup -- shipped 2026-08-28 (15/15). Sprint 8 (Open Items) still tracks FAQ sign-off, logo colour mismatch, GitHub Pages hosting, and post-Pages production deployment. Total: 70/74 (95%).</t>
         </is>
       </c>
       <c r="B3" s="18" t="inlineStr"/>
@@ -1393,6 +1457,39 @@
       <c r="G13" s="18" t="inlineStr">
         <is>
           <t>FAQ direction (awaiting sign-off), logo vs brand colour mismatch (flagged), GitHub Pages hosting (awaiting go-ahead), production deployment beyond Pages (deferred).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Sprint 9</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Hero v2 (layered parallax + video mockup)</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Three-plane hero: sunset bg + product-tour video card + desk fg, per-layer parallax + blur, right-to-left trust marquee, autoplay hardened. Supersedes S5-06 + S6-03.</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4554,6 +4651,786 @@
         </is>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.1</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>assets/img/hero-photo-v2.jpg</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="inlineStr">
+        <is>
+          <t>V2 hero image swap (sunset with figure)</t>
+        </is>
+      </c>
+      <c r="F61" s="18" t="inlineStr">
+        <is>
+          <t>Swapped the amber-wall guy hero for a sunset-mountain photo with a woman at a desk. Compressed source PNG (1.9MB) to hero-photo-v2.jpg (~240KB). Later superseded by V3 (people-free scene) so the composition would work equally well with the incoming foreground desk plane in front of it.</t>
+        </is>
+      </c>
+      <c r="G61" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H61" s="18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I61" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J61" s="18" t="inlineStr"/>
+      <c r="K61" s="18" t="inlineStr"/>
+      <c r="L61" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.2</t>
+        </is>
+      </c>
+      <c r="B62" s="18" t="inlineStr">
+        <is>
+          <t>assets/img/hero-bg.jpg</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>V3 background image (sunset valley, no figure)</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>Adopted the layered-source bottom image as the final hero background. Sunset over a mountain valley, no people, so the desk foreground reads as the viewer's own workspace. 323KB after sips-JPEG compression.</t>
+        </is>
+      </c>
+      <c r="G62" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H62" s="18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I62" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J62" s="18" t="inlineStr"/>
+      <c r="K62" s="18" t="inlineStr"/>
+      <c r="L62" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.3</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>assets/img/hero-fg.webp</t>
+        </is>
+      </c>
+      <c r="C63" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Foreground desk plane (alpha PNG -&gt; WebP)</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="inlineStr">
+        <is>
+          <t>Encoded the desk foreground with transparency (WebP 113KB with alpha, PNG 983KB fallback for old browsers). Positioned at z:3 so the desk edge sits in front of the video card, making the mockup feel like it's floating in the sky.</t>
+        </is>
+      </c>
+      <c r="G63" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I63" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J63" s="18" t="inlineStr"/>
+      <c r="K63" s="18" t="inlineStr"/>
+      <c r="L63" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.4</t>
+        </is>
+      </c>
+      <c r="B64" s="18" t="inlineStr">
+        <is>
+          <t>index.html, styles.css (planes)</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>Structure</t>
+        </is>
+      </c>
+      <c r="E64" s="18" t="inlineStr">
+        <is>
+          <t>Three-plane depth composition</t>
+        </is>
+      </c>
+      <c r="F64" s="18" t="inlineStr">
+        <is>
+          <t>Restructured the hero markup into hero-bg (z:0) + hero-content middle (z:2) + hero-fg (z:3). Cards and copy sit between the sky and the desk. isolation:isolate on .hero contains the stacking context.</t>
+        </is>
+      </c>
+      <c r="G64" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H64" s="18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I64" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J64" s="18" t="inlineStr"/>
+      <c r="K64" s="18" t="inlineStr"/>
+      <c r="L64" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.5</t>
+        </is>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
+          <t>assets/img/hero-mockup.{webm,mp4}</t>
+        </is>
+      </c>
+      <c r="C65" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D65" s="18" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E65" s="18" t="inlineStr">
+        <is>
+          <t>Product-tour video card replaces the 6-card grid</t>
+        </is>
+      </c>
+      <c r="F65" s="18" t="inlineStr">
+        <is>
+          <t>Removed the six static metric mockup cards. Replaced with a single curved card (clamp(12px,1.4vw,20px) radius, glass rim, 700px wide, ~1.87:1 aspect) playing the DecisionOS product tour on autoplay muted loop. Video source: Hero 2.mp4 re-encoded to WebM (997KB, VP9) + MP4 (768KB, H.264), audio stripped, 30fps.</t>
+        </is>
+      </c>
+      <c r="G65" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H65" s="18" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I65" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J65" s="18" t="inlineStr"/>
+      <c r="K65" s="18" t="inlineStr"/>
+      <c r="L65" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.6</t>
+        </is>
+      </c>
+      <c r="B66" s="18" t="inlineStr">
+        <is>
+          <t>assets/img/hero-mockup.*</t>
+        </is>
+      </c>
+      <c r="C66" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D66" s="18" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="E66" s="18" t="inlineStr">
+        <is>
+          <t>Video top-crop tuned to reveal mockup nav bar</t>
+        </is>
+      </c>
+      <c r="F66" s="18" t="inlineStr">
+        <is>
+          <t>Iterated the video crop: 12% top crop removed the browser chrome (URL bar) but also hid the DecisionOS product nav bar. Reduced to 5% top crop, which drops the browser Chrome while keeping the mockup's own nav (Decision Desk / My Work / Ops / CRM / ...) visible.</t>
+        </is>
+      </c>
+      <c r="G66" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H66" s="18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I66" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J66" s="18" t="inlineStr"/>
+      <c r="K66" s="18" t="inlineStr"/>
+      <c r="L66" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.7</t>
+        </is>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>index.html (autoplay script)</t>
+        </is>
+      </c>
+      <c r="C67" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D67" s="18" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E67" s="18" t="inlineStr">
+        <is>
+          <t>Autoplay hardened for policy-blocked browsers</t>
+        </is>
+      </c>
+      <c r="F67" s="18" t="inlineStr">
+        <is>
+          <t>Chrome's autoplay policy sometimes defers .play() past the initial DOMContentLoaded. Retries on loadedmetadata / loadeddata / canplay / canplaythrough / window.load, plus a 250ms poll for up to 6s. First user interaction (pointerdown) unblocks permanently.</t>
+        </is>
+      </c>
+      <c r="G67" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H67" s="18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I67" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J67" s="18" t="inlineStr"/>
+      <c r="K67" s="18" t="inlineStr"/>
+      <c r="L67" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.8</t>
+        </is>
+      </c>
+      <c r="B68" s="18" t="inlineStr">
+        <is>
+          <t>styles.css (parallax)</t>
+        </is>
+      </c>
+      <c r="C68" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D68" s="18" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E68" s="18" t="inlineStr">
+        <is>
+          <t>Per-layer parallax on scroll (no sticky pin)</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="inlineStr">
+        <is>
+          <t>Rebuilt the hero scroll model. Hero is position:relative (not sticky). As it scrolls, each layer counter-translates to lag behind the natural scroll at its own rate: bg 70vh (30% apparent speed), fg 0 (100% -- anchor), copy 30vh (70%), video card 32vh (68%), partners 45vh (55%). Layers slide past each other so the composition reads as three-dimensional depth. Uses the existing --hp scroll variable set by main.js Sprint 6.</t>
+        </is>
+      </c>
+      <c r="G68" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H68" s="18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I68" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J68" s="18" t="inlineStr"/>
+      <c r="K68" s="18" t="inlineStr"/>
+      <c r="L68" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.9</t>
+        </is>
+      </c>
+      <c r="B69" s="18" t="inlineStr">
+        <is>
+          <t>styles.css (parallax)</t>
+        </is>
+      </c>
+      <c r="C69" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D69" s="18" t="inlineStr">
+        <is>
+          <t>Motion</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="inlineStr">
+        <is>
+          <t>Independent blur curve per layer</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>Each parallax layer blurs at its own rate as --hp grows: bg 15px, fg 10px, copy 5px, video card 5px, trust band 10px. Softens the recede without pausing the video. prefers-reduced-motion: reduce disables both parallax and blur.</t>
+        </is>
+      </c>
+      <c r="G69" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H69" s="18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I69" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J69" s="18" t="inlineStr"/>
+      <c r="K69" s="18" t="inlineStr"/>
+      <c r="L69" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.10</t>
+        </is>
+      </c>
+      <c r="B70" s="18" t="inlineStr">
+        <is>
+          <t>styles.css (nav)</t>
+        </is>
+      </c>
+      <c r="C70" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D70" s="18" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="inlineStr">
+        <is>
+          <t>Nav bar always visible on hero (was hidden until scroll)</t>
+        </is>
+      </c>
+      <c r="F70" s="18" t="inlineStr">
+        <is>
+          <t>Removed the "swipe in from top when scrolled 55% of hero height" behaviour on .site-header. The nav is now visible from page load so the DecisionOS logo and links sit in the top-left the whole time, matching the reference mockup.</t>
+        </is>
+      </c>
+      <c r="G70" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H70" s="18" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I70" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J70" s="18" t="inlineStr"/>
+      <c r="K70" s="18" t="inlineStr"/>
+      <c r="L70" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.11</t>
+        </is>
+      </c>
+      <c r="B71" s="18" t="inlineStr">
+        <is>
+          <t>index.html, styles.css (trust band)</t>
+        </is>
+      </c>
+      <c r="C71" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D71" s="18" t="inlineStr">
+        <is>
+          <t>Content</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="inlineStr">
+        <is>
+          <t>Trust band as contained right-to-left marquee</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>Lifted the "Trusted by founder-led businesses" strip from the hero bottom (where the desk foreground was hiding it) into a mid-hero band. 780px wide, centred, positioned with balanced headroom above and below the video card. Brand list duplicated twice for a seamless 28s right-to-left loop with fade-edge mask-image on both sides.</t>
+        </is>
+      </c>
+      <c r="G71" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H71" s="18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I71" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J71" s="18" t="inlineStr"/>
+      <c r="K71" s="18" t="inlineStr"/>
+      <c r="L71" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.12</t>
+        </is>
+      </c>
+      <c r="B72" s="18" t="inlineStr">
+        <is>
+          <t>index.html (dex bubble)</t>
+        </is>
+      </c>
+      <c r="C72" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="inlineStr">
+        <is>
+          <t>Remove Dex bubble from hero</t>
+        </is>
+      </c>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>The Dex-today's-read floating callout was compact-styled once and then removed entirely -- the video card itself carries the "here's the product" moment.</t>
+        </is>
+      </c>
+      <c r="G72" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H72" s="18" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I72" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J72" s="18" t="inlineStr"/>
+      <c r="K72" s="18" t="inlineStr"/>
+      <c r="L72" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.13</t>
+        </is>
+      </c>
+      <c r="B73" s="18" t="inlineStr">
+        <is>
+          <t>index.html (scroll cue)</t>
+        </is>
+      </c>
+      <c r="C73" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D73" s="18" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="inlineStr">
+        <is>
+          <t>Remove scroll cue anchor</t>
+        </is>
+      </c>
+      <c r="F73" s="18" t="inlineStr">
+        <is>
+          <t>The scroll indicator at the bottom of the hero was removed. The composition already has enough motion to signal there's more below.</t>
+        </is>
+      </c>
+      <c r="G73" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H73" s="18" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I73" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J73" s="18" t="inlineStr"/>
+      <c r="K73" s="18" t="inlineStr"/>
+      <c r="L73" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.14</t>
+        </is>
+      </c>
+      <c r="B74" s="18" t="inlineStr">
+        <is>
+          <t>index.html (video card)</t>
+        </is>
+      </c>
+      <c r="C74" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D74" s="18" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="inlineStr">
+        <is>
+          <t>Fix: video card wasn't parallaxing (reveal class override)</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>.hero-video-card had class="reveal" whose fade-in animation runs with fill-mode:forwards, ending at transform:none. That fill-mode-held value silently overrode the per-layer parallax translate3d on the same element -- so it was the only middle-plane element not visibly moving on scroll. Dropped the reveal class from the video card (hero-copy and hero-partners carry reveal only on their children, so their parallax kept working).</t>
+        </is>
+      </c>
+      <c r="G74" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H74" s="18" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I74" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J74" s="18" t="inlineStr"/>
+      <c r="K74" s="18" t="inlineStr"/>
+      <c r="L74" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="inlineStr">
+        <is>
+          <t>U9-09.15</t>
+        </is>
+      </c>
+      <c r="B75" s="18" t="inlineStr">
+        <is>
+          <t>styles.css (trust band transform)</t>
+        </is>
+      </c>
+      <c r="C75" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D75" s="18" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="inlineStr">
+        <is>
+          <t>Fix: trust band centering + parallax translate3d fought each other</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="inlineStr">
+        <is>
+          <t>.hero-partners had two transform declarations -- translateX(-50%) for centering, and translate3d(...) for parallax. Second overrode the first, leaving the band 390px off-centre. Merged into a single transform: translate(-50%, calc(var(--hp)*45vh)) so it centres AND parallaxes.</t>
+        </is>
+      </c>
+      <c r="G75" s="18" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H75" s="18" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I75" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J75" s="18" t="inlineStr"/>
+      <c r="K75" s="18" t="inlineStr"/>
+      <c r="L75" s="18" t="inlineStr">
+        <is>
+          <t>commit 15b51cc (hero v10) + landing-page/landing-page-build-tracker.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>